<commit_message>
Updated output data ISIC 41T43
</commit_message>
<xml_diff>
--- a/InputData/io-model/BObIC/BAU Output by ISIC Code.xlsx
+++ b/InputData/io-model/BObIC/BAU Output by ISIC Code.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10526"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ssy02/Desktop/Postdoc Projects/eps-brazil-cpl/InputData/io-model/BObIC/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saido\OneDrive\Documents\eps-brazil-cpl\InputData\io-model\BObIC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EBB687B-A74A-7240-9325-DBB6CB0C6448}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21360" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -18,7 +17,7 @@
     <sheet name="BR Data for ISIC Splits" sheetId="10" r:id="rId3"/>
     <sheet name="BObIC" sheetId="2" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="152511" iterate="1" iterateDelta="1.0000000000000001E-5"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -734,7 +733,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="5">
     <numFmt numFmtId="164" formatCode="#,##0.0_ ;\-#,##0.0\ "/>
     <numFmt numFmtId="165" formatCode="0.000"/>
@@ -1371,7 +1370,6 @@
     <xf numFmtId="38" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="38" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1408,13 +1406,14 @@
     <xf numFmtId="0" fontId="17" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="11" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="5">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="2" xr:uid="{3ADF3FF5-E4D2-4BC8-9960-7408DCCB591E}"/>
-    <cellStyle name="Normal 4" xfId="4" xr:uid="{A9A180C4-0DBD-48FB-93F3-8D313F8559BC}"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Normal 2" xfId="2"/>
+    <cellStyle name="Normal 4" xfId="4"/>
+    <cellStyle name="Pourcentage" xfId="3" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1691,19 +1690,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B30"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="77.5" customWidth="1"/>
+    <col min="2" max="2" width="77.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -1711,117 +1710,117 @@
         <v>147</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B5" s="2">
         <v>2018</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" s="3" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B10" s="17" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B13" s="48" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B14" s="38" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B15" s="38" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B16" s="38" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="16">
         <v>0.9686815713640794</v>
       </c>
@@ -1831,8 +1830,8 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B7" r:id="rId1" xr:uid="{C914AE0B-59C0-465D-B416-7732EA12FF11}"/>
-    <hyperlink ref="A27" r:id="rId2" xr:uid="{4893E3FE-35AF-4F05-8AAC-FB415FA959C9}"/>
+    <hyperlink ref="B7" r:id="rId1"/>
+    <hyperlink ref="A27" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId3"/>
@@ -1840,27 +1839,27 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBC40CF3-8B3B-41DC-A935-B8F6C9564C97}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AU55"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="27.5" style="6" customWidth="1"/>
-    <col min="2" max="2" width="2.5" style="6" customWidth="1"/>
-    <col min="3" max="23" width="9.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="24" max="26" width="9.5" style="6" bestFit="1" customWidth="1"/>
-    <col min="27" max="30" width="9.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="31" max="36" width="9.5" style="6" bestFit="1" customWidth="1"/>
-    <col min="37" max="38" width="9.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="10.5" style="6" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="9.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="41" max="42" width="9.5" style="6" bestFit="1" customWidth="1"/>
-    <col min="43" max="45" width="9.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="9.5" style="6" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="10.1640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="48" max="16384" width="9.1640625" style="6"/>
+    <col min="1" max="1" width="27.42578125" style="6" customWidth="1"/>
+    <col min="2" max="2" width="2.42578125" style="6" customWidth="1"/>
+    <col min="3" max="23" width="9.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="24" max="26" width="9.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="27" max="30" width="9.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="31" max="36" width="9.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="37" max="38" width="9.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="10.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="9.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="41" max="42" width="9.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="43" max="45" width="9.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="9.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="10.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="48" max="16384" width="9.140625" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" hidden="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:47" hidden="1" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="e">
         <f ca="1">DotStatQuery(B1)</f>
         <v>#NAME?</v>
@@ -1869,228 +1868,228 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:47" ht="26" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:47" ht="23.25" x14ac:dyDescent="0.2">
       <c r="A2" s="7" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:47" x14ac:dyDescent="0.15">
-      <c r="A3" s="82" t="s">
+    <row r="3" spans="1:47" x14ac:dyDescent="0.2">
+      <c r="A3" s="81" t="s">
         <v>42</v>
       </c>
-      <c r="B3" s="83"/>
-      <c r="C3" s="89" t="s">
+      <c r="B3" s="82"/>
+      <c r="C3" s="88" t="s">
         <v>43</v>
       </c>
-      <c r="D3" s="90"/>
-      <c r="E3" s="90"/>
-      <c r="F3" s="90"/>
-      <c r="G3" s="90"/>
-      <c r="H3" s="90"/>
-      <c r="I3" s="90"/>
-      <c r="J3" s="90"/>
-      <c r="K3" s="90"/>
-      <c r="L3" s="90"/>
-      <c r="M3" s="90"/>
-      <c r="N3" s="90"/>
-      <c r="O3" s="90"/>
-      <c r="P3" s="90"/>
-      <c r="Q3" s="90"/>
-      <c r="R3" s="90"/>
-      <c r="S3" s="90"/>
-      <c r="T3" s="90"/>
-      <c r="U3" s="90"/>
-      <c r="V3" s="90"/>
-      <c r="W3" s="90"/>
-      <c r="X3" s="90"/>
-      <c r="Y3" s="90"/>
-      <c r="Z3" s="90"/>
-      <c r="AA3" s="90"/>
-      <c r="AB3" s="90"/>
-      <c r="AC3" s="90"/>
-      <c r="AD3" s="90"/>
-      <c r="AE3" s="90"/>
-      <c r="AF3" s="90"/>
-      <c r="AG3" s="90"/>
-      <c r="AH3" s="90"/>
-      <c r="AI3" s="90"/>
-      <c r="AJ3" s="90"/>
-      <c r="AK3" s="90"/>
-      <c r="AL3" s="90"/>
-      <c r="AM3" s="90"/>
-      <c r="AN3" s="90"/>
-      <c r="AO3" s="90"/>
-      <c r="AP3" s="90"/>
-      <c r="AQ3" s="90"/>
-      <c r="AR3" s="90"/>
-      <c r="AS3" s="90"/>
-      <c r="AT3" s="90"/>
-      <c r="AU3" s="91"/>
-    </row>
-    <row r="4" spans="1:47" x14ac:dyDescent="0.15">
-      <c r="A4" s="82" t="s">
+      <c r="D3" s="89"/>
+      <c r="E3" s="89"/>
+      <c r="F3" s="89"/>
+      <c r="G3" s="89"/>
+      <c r="H3" s="89"/>
+      <c r="I3" s="89"/>
+      <c r="J3" s="89"/>
+      <c r="K3" s="89"/>
+      <c r="L3" s="89"/>
+      <c r="M3" s="89"/>
+      <c r="N3" s="89"/>
+      <c r="O3" s="89"/>
+      <c r="P3" s="89"/>
+      <c r="Q3" s="89"/>
+      <c r="R3" s="89"/>
+      <c r="S3" s="89"/>
+      <c r="T3" s="89"/>
+      <c r="U3" s="89"/>
+      <c r="V3" s="89"/>
+      <c r="W3" s="89"/>
+      <c r="X3" s="89"/>
+      <c r="Y3" s="89"/>
+      <c r="Z3" s="89"/>
+      <c r="AA3" s="89"/>
+      <c r="AB3" s="89"/>
+      <c r="AC3" s="89"/>
+      <c r="AD3" s="89"/>
+      <c r="AE3" s="89"/>
+      <c r="AF3" s="89"/>
+      <c r="AG3" s="89"/>
+      <c r="AH3" s="89"/>
+      <c r="AI3" s="89"/>
+      <c r="AJ3" s="89"/>
+      <c r="AK3" s="89"/>
+      <c r="AL3" s="89"/>
+      <c r="AM3" s="89"/>
+      <c r="AN3" s="89"/>
+      <c r="AO3" s="89"/>
+      <c r="AP3" s="89"/>
+      <c r="AQ3" s="89"/>
+      <c r="AR3" s="89"/>
+      <c r="AS3" s="89"/>
+      <c r="AT3" s="89"/>
+      <c r="AU3" s="90"/>
+    </row>
+    <row r="4" spans="1:47" x14ac:dyDescent="0.2">
+      <c r="A4" s="81" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="83"/>
-      <c r="C4" s="84" t="s">
+      <c r="B4" s="82"/>
+      <c r="C4" s="83" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="85"/>
-      <c r="E4" s="85"/>
-      <c r="F4" s="85"/>
-      <c r="G4" s="85"/>
-      <c r="H4" s="85"/>
-      <c r="I4" s="85"/>
-      <c r="J4" s="85"/>
-      <c r="K4" s="85"/>
-      <c r="L4" s="85"/>
-      <c r="M4" s="85"/>
-      <c r="N4" s="85"/>
-      <c r="O4" s="85"/>
-      <c r="P4" s="85"/>
-      <c r="Q4" s="85"/>
-      <c r="R4" s="85"/>
-      <c r="S4" s="85"/>
-      <c r="T4" s="85"/>
-      <c r="U4" s="85"/>
-      <c r="V4" s="85"/>
-      <c r="W4" s="85"/>
-      <c r="X4" s="85"/>
-      <c r="Y4" s="85"/>
-      <c r="Z4" s="85"/>
-      <c r="AA4" s="85"/>
-      <c r="AB4" s="85"/>
-      <c r="AC4" s="85"/>
-      <c r="AD4" s="85"/>
-      <c r="AE4" s="85"/>
-      <c r="AF4" s="85"/>
-      <c r="AG4" s="85"/>
-      <c r="AH4" s="85"/>
-      <c r="AI4" s="85"/>
-      <c r="AJ4" s="85"/>
-      <c r="AK4" s="85"/>
-      <c r="AL4" s="85"/>
-      <c r="AM4" s="85"/>
-      <c r="AN4" s="85"/>
-      <c r="AO4" s="85"/>
-      <c r="AP4" s="85"/>
-      <c r="AQ4" s="85"/>
-      <c r="AR4" s="85"/>
-      <c r="AS4" s="85"/>
-      <c r="AT4" s="85"/>
-      <c r="AU4" s="86"/>
-    </row>
-    <row r="5" spans="1:47" x14ac:dyDescent="0.15">
-      <c r="A5" s="82" t="s">
+      <c r="D4" s="84"/>
+      <c r="E4" s="84"/>
+      <c r="F4" s="84"/>
+      <c r="G4" s="84"/>
+      <c r="H4" s="84"/>
+      <c r="I4" s="84"/>
+      <c r="J4" s="84"/>
+      <c r="K4" s="84"/>
+      <c r="L4" s="84"/>
+      <c r="M4" s="84"/>
+      <c r="N4" s="84"/>
+      <c r="O4" s="84"/>
+      <c r="P4" s="84"/>
+      <c r="Q4" s="84"/>
+      <c r="R4" s="84"/>
+      <c r="S4" s="84"/>
+      <c r="T4" s="84"/>
+      <c r="U4" s="84"/>
+      <c r="V4" s="84"/>
+      <c r="W4" s="84"/>
+      <c r="X4" s="84"/>
+      <c r="Y4" s="84"/>
+      <c r="Z4" s="84"/>
+      <c r="AA4" s="84"/>
+      <c r="AB4" s="84"/>
+      <c r="AC4" s="84"/>
+      <c r="AD4" s="84"/>
+      <c r="AE4" s="84"/>
+      <c r="AF4" s="84"/>
+      <c r="AG4" s="84"/>
+      <c r="AH4" s="84"/>
+      <c r="AI4" s="84"/>
+      <c r="AJ4" s="84"/>
+      <c r="AK4" s="84"/>
+      <c r="AL4" s="84"/>
+      <c r="AM4" s="84"/>
+      <c r="AN4" s="84"/>
+      <c r="AO4" s="84"/>
+      <c r="AP4" s="84"/>
+      <c r="AQ4" s="84"/>
+      <c r="AR4" s="84"/>
+      <c r="AS4" s="84"/>
+      <c r="AT4" s="84"/>
+      <c r="AU4" s="85"/>
+    </row>
+    <row r="5" spans="1:47" x14ac:dyDescent="0.2">
+      <c r="A5" s="81" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="83"/>
-      <c r="C5" s="84" t="s">
+      <c r="B5" s="82"/>
+      <c r="C5" s="83" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="85"/>
-      <c r="E5" s="85"/>
-      <c r="F5" s="85"/>
-      <c r="G5" s="85"/>
-      <c r="H5" s="85"/>
-      <c r="I5" s="85"/>
-      <c r="J5" s="85"/>
-      <c r="K5" s="85"/>
-      <c r="L5" s="85"/>
-      <c r="M5" s="85"/>
-      <c r="N5" s="85"/>
-      <c r="O5" s="85"/>
-      <c r="P5" s="85"/>
-      <c r="Q5" s="85"/>
-      <c r="R5" s="85"/>
-      <c r="S5" s="85"/>
-      <c r="T5" s="85"/>
-      <c r="U5" s="85"/>
-      <c r="V5" s="85"/>
-      <c r="W5" s="85"/>
-      <c r="X5" s="85"/>
-      <c r="Y5" s="85"/>
-      <c r="Z5" s="85"/>
-      <c r="AA5" s="85"/>
-      <c r="AB5" s="85"/>
-      <c r="AC5" s="85"/>
-      <c r="AD5" s="85"/>
-      <c r="AE5" s="85"/>
-      <c r="AF5" s="85"/>
-      <c r="AG5" s="85"/>
-      <c r="AH5" s="85"/>
-      <c r="AI5" s="85"/>
-      <c r="AJ5" s="85"/>
-      <c r="AK5" s="85"/>
-      <c r="AL5" s="85"/>
-      <c r="AM5" s="85"/>
-      <c r="AN5" s="85"/>
-      <c r="AO5" s="85"/>
-      <c r="AP5" s="85"/>
-      <c r="AQ5" s="85"/>
-      <c r="AR5" s="85"/>
-      <c r="AS5" s="85"/>
-      <c r="AT5" s="85"/>
-      <c r="AU5" s="86"/>
-    </row>
-    <row r="6" spans="1:47" x14ac:dyDescent="0.15">
-      <c r="A6" s="82" t="s">
+      <c r="D5" s="84"/>
+      <c r="E5" s="84"/>
+      <c r="F5" s="84"/>
+      <c r="G5" s="84"/>
+      <c r="H5" s="84"/>
+      <c r="I5" s="84"/>
+      <c r="J5" s="84"/>
+      <c r="K5" s="84"/>
+      <c r="L5" s="84"/>
+      <c r="M5" s="84"/>
+      <c r="N5" s="84"/>
+      <c r="O5" s="84"/>
+      <c r="P5" s="84"/>
+      <c r="Q5" s="84"/>
+      <c r="R5" s="84"/>
+      <c r="S5" s="84"/>
+      <c r="T5" s="84"/>
+      <c r="U5" s="84"/>
+      <c r="V5" s="84"/>
+      <c r="W5" s="84"/>
+      <c r="X5" s="84"/>
+      <c r="Y5" s="84"/>
+      <c r="Z5" s="84"/>
+      <c r="AA5" s="84"/>
+      <c r="AB5" s="84"/>
+      <c r="AC5" s="84"/>
+      <c r="AD5" s="84"/>
+      <c r="AE5" s="84"/>
+      <c r="AF5" s="84"/>
+      <c r="AG5" s="84"/>
+      <c r="AH5" s="84"/>
+      <c r="AI5" s="84"/>
+      <c r="AJ5" s="84"/>
+      <c r="AK5" s="84"/>
+      <c r="AL5" s="84"/>
+      <c r="AM5" s="84"/>
+      <c r="AN5" s="84"/>
+      <c r="AO5" s="84"/>
+      <c r="AP5" s="84"/>
+      <c r="AQ5" s="84"/>
+      <c r="AR5" s="84"/>
+      <c r="AS5" s="84"/>
+      <c r="AT5" s="84"/>
+      <c r="AU5" s="85"/>
+    </row>
+    <row r="6" spans="1:47" x14ac:dyDescent="0.2">
+      <c r="A6" s="81" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="83"/>
-      <c r="C6" s="84" t="s">
+      <c r="B6" s="82"/>
+      <c r="C6" s="83" t="s">
         <v>44</v>
       </c>
-      <c r="D6" s="85"/>
-      <c r="E6" s="85"/>
-      <c r="F6" s="85"/>
-      <c r="G6" s="85"/>
-      <c r="H6" s="85"/>
-      <c r="I6" s="85"/>
-      <c r="J6" s="85"/>
-      <c r="K6" s="85"/>
-      <c r="L6" s="85"/>
-      <c r="M6" s="85"/>
-      <c r="N6" s="85"/>
-      <c r="O6" s="85"/>
-      <c r="P6" s="85"/>
-      <c r="Q6" s="85"/>
-      <c r="R6" s="85"/>
-      <c r="S6" s="85"/>
-      <c r="T6" s="85"/>
-      <c r="U6" s="85"/>
-      <c r="V6" s="85"/>
-      <c r="W6" s="85"/>
-      <c r="X6" s="85"/>
-      <c r="Y6" s="85"/>
-      <c r="Z6" s="85"/>
-      <c r="AA6" s="85"/>
-      <c r="AB6" s="85"/>
-      <c r="AC6" s="85"/>
-      <c r="AD6" s="85"/>
-      <c r="AE6" s="85"/>
-      <c r="AF6" s="85"/>
-      <c r="AG6" s="85"/>
-      <c r="AH6" s="85"/>
-      <c r="AI6" s="85"/>
-      <c r="AJ6" s="85"/>
-      <c r="AK6" s="85"/>
-      <c r="AL6" s="85"/>
-      <c r="AM6" s="85"/>
-      <c r="AN6" s="85"/>
-      <c r="AO6" s="85"/>
-      <c r="AP6" s="85"/>
-      <c r="AQ6" s="85"/>
-      <c r="AR6" s="85"/>
-      <c r="AS6" s="85"/>
-      <c r="AT6" s="85"/>
-      <c r="AU6" s="86"/>
-    </row>
-    <row r="7" spans="1:47" ht="120" x14ac:dyDescent="0.15">
-      <c r="A7" s="87" t="s">
+      <c r="D6" s="84"/>
+      <c r="E6" s="84"/>
+      <c r="F6" s="84"/>
+      <c r="G6" s="84"/>
+      <c r="H6" s="84"/>
+      <c r="I6" s="84"/>
+      <c r="J6" s="84"/>
+      <c r="K6" s="84"/>
+      <c r="L6" s="84"/>
+      <c r="M6" s="84"/>
+      <c r="N6" s="84"/>
+      <c r="O6" s="84"/>
+      <c r="P6" s="84"/>
+      <c r="Q6" s="84"/>
+      <c r="R6" s="84"/>
+      <c r="S6" s="84"/>
+      <c r="T6" s="84"/>
+      <c r="U6" s="84"/>
+      <c r="V6" s="84"/>
+      <c r="W6" s="84"/>
+      <c r="X6" s="84"/>
+      <c r="Y6" s="84"/>
+      <c r="Z6" s="84"/>
+      <c r="AA6" s="84"/>
+      <c r="AB6" s="84"/>
+      <c r="AC6" s="84"/>
+      <c r="AD6" s="84"/>
+      <c r="AE6" s="84"/>
+      <c r="AF6" s="84"/>
+      <c r="AG6" s="84"/>
+      <c r="AH6" s="84"/>
+      <c r="AI6" s="84"/>
+      <c r="AJ6" s="84"/>
+      <c r="AK6" s="84"/>
+      <c r="AL6" s="84"/>
+      <c r="AM6" s="84"/>
+      <c r="AN6" s="84"/>
+      <c r="AO6" s="84"/>
+      <c r="AP6" s="84"/>
+      <c r="AQ6" s="84"/>
+      <c r="AR6" s="84"/>
+      <c r="AS6" s="84"/>
+      <c r="AT6" s="84"/>
+      <c r="AU6" s="85"/>
+    </row>
+    <row r="7" spans="1:47" ht="126" x14ac:dyDescent="0.2">
+      <c r="A7" s="86" t="s">
         <v>45</v>
       </c>
-      <c r="B7" s="88"/>
+      <c r="B7" s="87"/>
       <c r="C7" s="8" t="s">
         <v>46</v>
       </c>
@@ -2227,7 +2226,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="8" spans="1:47" ht="14" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:47" ht="13.5" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>91</v>
       </c>
@@ -2370,7 +2369,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:47" ht="24" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:47" ht="21" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
         <v>92</v>
       </c>
@@ -2513,7 +2512,7 @@
         <v>-37816</v>
       </c>
     </row>
-    <row r="10" spans="1:47" ht="24" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:47" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
         <v>93</v>
       </c>
@@ -2656,7 +2655,7 @@
         <v>-161022.9</v>
       </c>
     </row>
-    <row r="11" spans="1:47" ht="24" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:47" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
         <v>94</v>
       </c>
@@ -2799,7 +2798,7 @@
         <v>-7908.2</v>
       </c>
     </row>
-    <row r="12" spans="1:47" ht="24" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:47" ht="21" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
         <v>95</v>
       </c>
@@ -2942,7 +2941,7 @@
         <v>-1554.4</v>
       </c>
     </row>
-    <row r="13" spans="1:47" ht="24" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:47" ht="21" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
         <v>96</v>
       </c>
@@ -3085,7 +3084,7 @@
         <v>-84486.2</v>
       </c>
     </row>
-    <row r="14" spans="1:47" ht="24" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:47" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
         <v>97</v>
       </c>
@@ -3228,7 +3227,7 @@
         <v>-145065.5</v>
       </c>
     </row>
-    <row r="15" spans="1:47" ht="24" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:47" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
         <v>98</v>
       </c>
@@ -3371,7 +3370,7 @@
         <v>-16997.3</v>
       </c>
     </row>
-    <row r="16" spans="1:47" ht="24" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:47" ht="21" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
         <v>99</v>
       </c>
@@ -3514,7 +3513,7 @@
         <v>-23813.7</v>
       </c>
     </row>
-    <row r="17" spans="1:47" ht="24" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:47" ht="21" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
         <v>100</v>
       </c>
@@ -3657,7 +3656,7 @@
         <v>-55734.3</v>
       </c>
     </row>
-    <row r="18" spans="1:47" ht="24" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:47" ht="21" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
         <v>101</v>
       </c>
@@ -3800,7 +3799,7 @@
         <v>-165140.70000000001</v>
       </c>
     </row>
-    <row r="19" spans="1:47" ht="14" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:47" ht="21" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
         <v>102</v>
       </c>
@@ -3943,7 +3942,7 @@
         <v>-49527.3</v>
       </c>
     </row>
-    <row r="20" spans="1:47" ht="24" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:47" ht="21" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
         <v>103</v>
       </c>
@@ -4086,7 +4085,7 @@
         <v>-26110.400000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:47" ht="14" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:47" ht="21" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
         <v>104</v>
       </c>
@@ -4229,7 +4228,7 @@
         <v>-77529.899999999994</v>
       </c>
     </row>
-    <row r="22" spans="1:47" ht="24" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:47" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
         <v>105</v>
       </c>
@@ -4372,7 +4371,7 @@
         <v>-65502.400000000001</v>
       </c>
     </row>
-    <row r="23" spans="1:47" ht="24" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:47" ht="21" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
         <v>106</v>
       </c>
@@ -4515,7 +4514,7 @@
         <v>-240846.5</v>
       </c>
     </row>
-    <row r="24" spans="1:47" ht="14" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:47" ht="13.5" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
         <v>107</v>
       </c>
@@ -4658,7 +4657,7 @@
         <v>-88431.1</v>
       </c>
     </row>
-    <row r="25" spans="1:47" ht="24" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:47" ht="21" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
         <v>108</v>
       </c>
@@ -4801,7 +4800,7 @@
         <v>-128475.8</v>
       </c>
     </row>
-    <row r="26" spans="1:47" ht="24" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:47" ht="21" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
         <v>109</v>
       </c>
@@ -4944,7 +4943,7 @@
         <v>-306727.09999999998</v>
       </c>
     </row>
-    <row r="27" spans="1:47" ht="14" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:47" ht="21" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
         <v>110</v>
       </c>
@@ -5087,7 +5086,7 @@
         <v>-61444.6</v>
       </c>
     </row>
-    <row r="28" spans="1:47" ht="36" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:47" ht="42" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
         <v>111</v>
       </c>
@@ -5230,7 +5229,7 @@
         <v>-99643.3</v>
       </c>
     </row>
-    <row r="29" spans="1:47" ht="36" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:47" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
         <v>112</v>
       </c>
@@ -5373,7 +5372,7 @@
         <v>-4933</v>
       </c>
     </row>
-    <row r="30" spans="1:47" ht="14" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:47" ht="13.5" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
         <v>113</v>
       </c>
@@ -5516,7 +5515,7 @@
         <v>-1563</v>
       </c>
     </row>
-    <row r="31" spans="1:47" ht="24" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:47" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A31" s="11" t="s">
         <v>114</v>
       </c>
@@ -5659,7 +5658,7 @@
         <v>-197714.9</v>
       </c>
     </row>
-    <row r="32" spans="1:47" ht="24" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:47" ht="21" x14ac:dyDescent="0.25">
       <c r="A32" s="11" t="s">
         <v>115</v>
       </c>
@@ -5802,7 +5801,7 @@
         <v>-127601.9</v>
       </c>
     </row>
-    <row r="33" spans="1:47" ht="24" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:47" ht="21" x14ac:dyDescent="0.25">
       <c r="A33" s="11" t="s">
         <v>116</v>
       </c>
@@ -5945,7 +5944,7 @@
         <v>-51797.3</v>
       </c>
     </row>
-    <row r="34" spans="1:47" ht="24" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:47" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A34" s="11" t="s">
         <v>117</v>
       </c>
@@ -6088,7 +6087,7 @@
         <v>-11993.5</v>
       </c>
     </row>
-    <row r="35" spans="1:47" ht="14" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:47" ht="13.5" x14ac:dyDescent="0.25">
       <c r="A35" s="11" t="s">
         <v>118</v>
       </c>
@@ -6231,7 +6230,7 @@
         <v>-3766.8</v>
       </c>
     </row>
-    <row r="36" spans="1:47" ht="24" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:47" ht="21" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
         <v>119</v>
       </c>
@@ -6374,7 +6373,7 @@
         <v>-62979.199999999997</v>
       </c>
     </row>
-    <row r="37" spans="1:47" ht="24" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:47" ht="21" x14ac:dyDescent="0.25">
       <c r="A37" s="11" t="s">
         <v>120</v>
       </c>
@@ -6517,7 +6516,7 @@
         <v>-56936.7</v>
       </c>
     </row>
-    <row r="38" spans="1:47" ht="14" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:47" ht="13.5" x14ac:dyDescent="0.25">
       <c r="A38" s="11" t="s">
         <v>121</v>
       </c>
@@ -6660,7 +6659,7 @@
         <v>-10003</v>
       </c>
     </row>
-    <row r="39" spans="1:47" ht="24" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:47" ht="21" x14ac:dyDescent="0.25">
       <c r="A39" s="11" t="s">
         <v>122</v>
       </c>
@@ -6803,7 +6802,7 @@
         <v>-132575.6</v>
       </c>
     </row>
-    <row r="40" spans="1:47" ht="24" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:47" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A40" s="11" t="s">
         <v>123</v>
       </c>
@@ -6946,7 +6945,7 @@
         <v>-2410.8000000000002</v>
       </c>
     </row>
-    <row r="41" spans="1:47" ht="14" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:47" ht="13.5" x14ac:dyDescent="0.25">
       <c r="A41" s="11" t="s">
         <v>124</v>
       </c>
@@ -7089,7 +7088,7 @@
         <v>-11121.3</v>
       </c>
     </row>
-    <row r="42" spans="1:47" ht="24" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:47" ht="21" x14ac:dyDescent="0.25">
       <c r="A42" s="11" t="s">
         <v>125</v>
       </c>
@@ -7232,7 +7231,7 @@
         <v>-2867.1</v>
       </c>
     </row>
-    <row r="43" spans="1:47" ht="24" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:47" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A43" s="11" t="s">
         <v>126</v>
       </c>
@@ -7375,7 +7374,7 @@
         <v>-8872.6</v>
       </c>
     </row>
-    <row r="44" spans="1:47" ht="24" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:47" ht="21" x14ac:dyDescent="0.25">
       <c r="A44" s="11" t="s">
         <v>127</v>
       </c>
@@ -7518,7 +7517,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:47" ht="36" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:47" ht="42" x14ac:dyDescent="0.25">
       <c r="A45" s="11" t="s">
         <v>128</v>
       </c>
@@ -7661,7 +7660,7 @@
         <v>-52880.800000000003</v>
       </c>
     </row>
-    <row r="46" spans="1:47" ht="48" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:47" ht="52.5" x14ac:dyDescent="0.25">
       <c r="A46" s="11" t="s">
         <v>129</v>
       </c>
@@ -7804,7 +7803,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:47" ht="24" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:47" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A47" s="11" t="s">
         <v>130</v>
       </c>
@@ -7947,7 +7946,7 @@
         <v>-2583795.2000000002</v>
       </c>
     </row>
-    <row r="48" spans="1:47" ht="14" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:47" ht="21" x14ac:dyDescent="0.25">
       <c r="A48" s="11" t="s">
         <v>131</v>
       </c>
@@ -8090,7 +8089,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:47" ht="14" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:47" ht="13.5" x14ac:dyDescent="0.25">
       <c r="A49" s="11" t="s">
         <v>132</v>
       </c>
@@ -8233,20 +8232,20 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:47" x14ac:dyDescent="0.15">
+    <row r="50" spans="1:47" x14ac:dyDescent="0.2">
       <c r="A50" s="14" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="54" spans="1:47" ht="15" x14ac:dyDescent="0.2">
-      <c r="A54" s="81" t="s">
+    <row r="54" spans="1:47" ht="15" x14ac:dyDescent="0.25">
+      <c r="A54" s="80" t="s">
         <v>26</v>
       </c>
       <c r="C54" s="6" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="55" spans="1:47" ht="15" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:47" ht="15" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
         <v>230</v>
       </c>
@@ -8264,10 +8263,10 @@
     <mergeCell ref="C5:AU5"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" display="http://localhost/OECDStat_Metadata/ShowMetadata.ashx?Dataset=IOTSI4_2018&amp;ShowOnWeb=true&amp;Lang=en" xr:uid="{D1C4AACA-BBF4-43A5-880C-7C65E754CE2A}"/>
-    <hyperlink ref="C3" r:id="rId2" display="http://localhost/OECDStat_Metadata/ShowMetadata.ashx?Dataset=IOTSI4_2018&amp;Coords=[VAR].[TTL]&amp;ShowOnWeb=true&amp;Lang=en" xr:uid="{42F580DE-8495-4BA9-90EA-2C61139986C1}"/>
-    <hyperlink ref="A50" r:id="rId3" display="https://stats-3.oecd.org/index.aspx?DatasetCode=IOTSI4_2018" xr:uid="{D8DFEA93-7AED-4372-9474-6BEC5C03AEE9}"/>
-    <hyperlink ref="A55" r:id="rId4" xr:uid="{561CE503-307A-E748-A542-52EE6465E6BF}"/>
+    <hyperlink ref="A2" r:id="rId1" display="http://localhost/OECDStat_Metadata/ShowMetadata.ashx?Dataset=IOTSI4_2018&amp;ShowOnWeb=true&amp;Lang=en"/>
+    <hyperlink ref="C3" r:id="rId2" display="http://localhost/OECDStat_Metadata/ShowMetadata.ashx?Dataset=IOTSI4_2018&amp;Coords=[VAR].[TTL]&amp;ShowOnWeb=true&amp;Lang=en"/>
+    <hyperlink ref="A50" r:id="rId3" display="https://stats-3.oecd.org/index.aspx?DatasetCode=IOTSI4_2018"/>
+    <hyperlink ref="A55" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -8275,39 +8274,39 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0339536F-9934-4689-98A8-C778F8365AC3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:S23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="48.33203125" customWidth="1"/>
-    <col min="2" max="2" width="21.6640625" customWidth="1"/>
-    <col min="3" max="3" width="40.1640625" customWidth="1"/>
-    <col min="4" max="4" width="20.33203125" customWidth="1"/>
-    <col min="5" max="5" width="24.1640625" customWidth="1"/>
-    <col min="6" max="6" width="21.5" customWidth="1"/>
-    <col min="7" max="9" width="20.83203125" customWidth="1"/>
-    <col min="10" max="10" width="19.83203125" customWidth="1"/>
-    <col min="11" max="11" width="23.5" customWidth="1"/>
-    <col min="12" max="12" width="22.5" customWidth="1"/>
-    <col min="13" max="13" width="20.33203125" customWidth="1"/>
-    <col min="14" max="15" width="18.5" customWidth="1"/>
+    <col min="1" max="1" width="48.28515625" customWidth="1"/>
+    <col min="2" max="2" width="21.7109375" customWidth="1"/>
+    <col min="3" max="3" width="40.140625" customWidth="1"/>
+    <col min="4" max="4" width="20.28515625" customWidth="1"/>
+    <col min="5" max="5" width="24.140625" customWidth="1"/>
+    <col min="6" max="6" width="21.42578125" customWidth="1"/>
+    <col min="7" max="9" width="20.85546875" customWidth="1"/>
+    <col min="10" max="10" width="19.85546875" customWidth="1"/>
+    <col min="11" max="11" width="23.42578125" customWidth="1"/>
+    <col min="12" max="12" width="22.42578125" customWidth="1"/>
+    <col min="13" max="13" width="20.28515625" customWidth="1"/>
+    <col min="14" max="15" width="18.42578125" customWidth="1"/>
     <col min="16" max="16" width="23" customWidth="1"/>
-    <col min="17" max="17" width="20.83203125" customWidth="1"/>
-    <col min="18" max="18" width="19.1640625" customWidth="1"/>
-    <col min="19" max="19" width="16.5" customWidth="1"/>
+    <col min="17" max="17" width="20.85546875" customWidth="1"/>
+    <col min="18" max="18" width="19.140625" customWidth="1"/>
+    <col min="19" max="19" width="16.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" s="19" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="3" spans="1:19" s="24" customFormat="1" ht="33" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" s="24" customFormat="1" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="20" t="s">
         <v>162</v>
       </c>
@@ -8366,7 +8365,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="16" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:19" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
         <v>155</v>
       </c>
@@ -8417,7 +8416,7 @@
       </c>
       <c r="S4" s="52"/>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="25" t="s">
         <v>156</v>
       </c>
@@ -8471,7 +8470,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="28" t="s">
         <v>184</v>
       </c>
@@ -8534,7 +8533,7 @@
       </c>
       <c r="S6" s="25"/>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B8" s="39" t="s">
         <v>217</v>
       </c>
@@ -8546,7 +8545,7 @@
       <c r="F8" s="42"/>
       <c r="G8" s="40"/>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:19" ht="24" x14ac:dyDescent="0.25">
       <c r="B9" s="62">
         <v>580</v>
       </c>
@@ -8560,7 +8559,7 @@
       <c r="F9" s="40"/>
       <c r="G9" s="40"/>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:19" ht="24" x14ac:dyDescent="0.25">
       <c r="B10" s="63">
         <v>680</v>
       </c>
@@ -8574,7 +8573,7 @@
       <c r="F10" s="40"/>
       <c r="G10" s="40"/>
     </row>
-    <row r="11" spans="1:19" ht="26" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:19" ht="24" x14ac:dyDescent="0.25">
       <c r="B11" s="63">
         <v>791</v>
       </c>
@@ -8588,7 +8587,7 @@
       <c r="F11" s="40"/>
       <c r="G11" s="40"/>
     </row>
-    <row r="12" spans="1:19" ht="26" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:19" ht="24" x14ac:dyDescent="0.25">
       <c r="B12" s="64">
         <v>792</v>
       </c>
@@ -8602,7 +8601,7 @@
       <c r="F12" s="40"/>
       <c r="G12" s="40"/>
     </row>
-    <row r="13" spans="1:19" ht="26" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:19" ht="24" x14ac:dyDescent="0.25">
       <c r="B13" s="55">
         <v>2091</v>
       </c>
@@ -8616,7 +8615,7 @@
       <c r="F13" s="40"/>
       <c r="G13" s="40"/>
     </row>
-    <row r="14" spans="1:19" ht="26" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:19" ht="24" x14ac:dyDescent="0.25">
       <c r="B14" s="58">
         <v>2092</v>
       </c>
@@ -8630,7 +8629,7 @@
       <c r="F14" s="40"/>
       <c r="G14" s="40"/>
     </row>
-    <row r="15" spans="1:19" ht="26" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:19" ht="24" x14ac:dyDescent="0.25">
       <c r="B15" s="58">
         <v>2093</v>
       </c>
@@ -8644,7 +8643,7 @@
       <c r="F15" s="40"/>
       <c r="G15" s="40"/>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:19" ht="24" x14ac:dyDescent="0.25">
       <c r="B16" s="60">
         <v>2100</v>
       </c>
@@ -8658,7 +8657,7 @@
       <c r="F16" s="40"/>
       <c r="G16" s="40"/>
     </row>
-    <row r="17" spans="2:7" ht="26" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:7" ht="36" x14ac:dyDescent="0.25">
       <c r="B17" s="65">
         <v>2300</v>
       </c>
@@ -8679,7 +8678,7 @@
         <v>87114</v>
       </c>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:7" ht="24" x14ac:dyDescent="0.25">
       <c r="B18" s="68" t="s">
         <v>207</v>
       </c>
@@ -8700,7 +8699,7 @@
         <v>16383</v>
       </c>
     </row>
-    <row r="19" spans="2:7" ht="26" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:7" ht="24" x14ac:dyDescent="0.25">
       <c r="B19" s="71">
         <v>23003</v>
       </c>
@@ -8721,7 +8720,7 @@
         <v>24171</v>
       </c>
     </row>
-    <row r="20" spans="2:7" ht="26" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:7" ht="36" x14ac:dyDescent="0.25">
       <c r="B20" s="62">
         <v>2491</v>
       </c>
@@ -8741,7 +8740,7 @@
         <v>46560</v>
       </c>
     </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:7" ht="24" x14ac:dyDescent="0.25">
       <c r="B21" s="64">
         <v>2492</v>
       </c>
@@ -8755,7 +8754,7 @@
       <c r="F21" s="40"/>
       <c r="G21" s="40"/>
     </row>
-    <row r="22" spans="2:7" ht="26" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:7" ht="24" x14ac:dyDescent="0.25">
       <c r="B22" s="74">
         <v>3500</v>
       </c>
@@ -8765,7 +8764,7 @@
       <c r="D22" s="76">
         <v>175287.99999999997</v>
       </c>
-      <c r="E22" s="92" t="s">
+      <c r="E22" s="91" t="s">
         <v>215</v>
       </c>
       <c r="F22" s="46" t="s">
@@ -8775,7 +8774,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="23" spans="2:7" ht="26" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:7" ht="24" x14ac:dyDescent="0.25">
       <c r="B23" s="64">
         <v>3680</v>
       </c>
@@ -8785,7 +8784,7 @@
       <c r="D23" s="61">
         <v>25127</v>
       </c>
-      <c r="E23" s="92"/>
+      <c r="E23" s="91"/>
       <c r="F23" s="46" t="s">
         <v>176</v>
       </c>
@@ -8803,20 +8802,20 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor theme="8" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:AQ2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.1640625" customWidth="1"/>
-    <col min="2" max="26" width="10.1640625" customWidth="1"/>
-    <col min="27" max="27" width="12.83203125" customWidth="1"/>
-    <col min="28" max="43" width="10.1640625" customWidth="1"/>
+    <col min="1" max="1" width="20.140625" customWidth="1"/>
+    <col min="2" max="26" width="10.140625" customWidth="1"/>
+    <col min="27" max="27" width="12.85546875" customWidth="1"/>
+    <col min="28" max="43" width="10.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" s="4" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:43" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="15" t="s">
         <v>139</v>
       </c>
@@ -8901,7 +8900,7 @@
       <c r="AB1" s="31" t="s">
         <v>192</v>
       </c>
-      <c r="AC1" s="81" t="s">
+      <c r="AC1" s="80" t="s">
         <v>26</v>
       </c>
       <c r="AD1" s="4" t="s">
@@ -8947,7 +8946,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:43" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:43" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>140</v>
       </c>
@@ -9059,8 +9058,9 @@
         <f>'OECD TTL'!W49*10^6*About!$A$30*('BR Data for ISIC Splits'!R6/SUM('BR Data for ISIC Splits'!P6:R6))</f>
         <v>57763254487.389854</v>
       </c>
-      <c r="AC2" s="80">
-        <v>40309373273311.203</v>
+      <c r="AC2" s="92">
+        <f>'OECD TTL'!X30*10^6*About!A30</f>
+        <v>132321902.64833325</v>
       </c>
       <c r="AD2">
         <f>'OECD TTL'!Y49*10^6*About!$A$30</f>

</xml_diff>

<commit_message>
Updated output data for ISIC 41T43
</commit_message>
<xml_diff>
--- a/InputData/io-model/BObIC/BAU Output by ISIC Code.xlsx
+++ b/InputData/io-model/BObIC/BAU Output by ISIC Code.xlsx
@@ -1373,6 +1373,7 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="11" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
@@ -1406,7 +1407,6 @@
     <xf numFmtId="0" fontId="17" fillId="9" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="11" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
@@ -1874,222 +1874,222 @@
       </c>
     </row>
     <row r="3" spans="1:47" x14ac:dyDescent="0.2">
-      <c r="A3" s="81" t="s">
+      <c r="A3" s="82" t="s">
         <v>42</v>
       </c>
-      <c r="B3" s="82"/>
-      <c r="C3" s="88" t="s">
+      <c r="B3" s="83"/>
+      <c r="C3" s="89" t="s">
         <v>43</v>
       </c>
-      <c r="D3" s="89"/>
-      <c r="E3" s="89"/>
-      <c r="F3" s="89"/>
-      <c r="G3" s="89"/>
-      <c r="H3" s="89"/>
-      <c r="I3" s="89"/>
-      <c r="J3" s="89"/>
-      <c r="K3" s="89"/>
-      <c r="L3" s="89"/>
-      <c r="M3" s="89"/>
-      <c r="N3" s="89"/>
-      <c r="O3" s="89"/>
-      <c r="P3" s="89"/>
-      <c r="Q3" s="89"/>
-      <c r="R3" s="89"/>
-      <c r="S3" s="89"/>
-      <c r="T3" s="89"/>
-      <c r="U3" s="89"/>
-      <c r="V3" s="89"/>
-      <c r="W3" s="89"/>
-      <c r="X3" s="89"/>
-      <c r="Y3" s="89"/>
-      <c r="Z3" s="89"/>
-      <c r="AA3" s="89"/>
-      <c r="AB3" s="89"/>
-      <c r="AC3" s="89"/>
-      <c r="AD3" s="89"/>
-      <c r="AE3" s="89"/>
-      <c r="AF3" s="89"/>
-      <c r="AG3" s="89"/>
-      <c r="AH3" s="89"/>
-      <c r="AI3" s="89"/>
-      <c r="AJ3" s="89"/>
-      <c r="AK3" s="89"/>
-      <c r="AL3" s="89"/>
-      <c r="AM3" s="89"/>
-      <c r="AN3" s="89"/>
-      <c r="AO3" s="89"/>
-      <c r="AP3" s="89"/>
-      <c r="AQ3" s="89"/>
-      <c r="AR3" s="89"/>
-      <c r="AS3" s="89"/>
-      <c r="AT3" s="89"/>
-      <c r="AU3" s="90"/>
+      <c r="D3" s="90"/>
+      <c r="E3" s="90"/>
+      <c r="F3" s="90"/>
+      <c r="G3" s="90"/>
+      <c r="H3" s="90"/>
+      <c r="I3" s="90"/>
+      <c r="J3" s="90"/>
+      <c r="K3" s="90"/>
+      <c r="L3" s="90"/>
+      <c r="M3" s="90"/>
+      <c r="N3" s="90"/>
+      <c r="O3" s="90"/>
+      <c r="P3" s="90"/>
+      <c r="Q3" s="90"/>
+      <c r="R3" s="90"/>
+      <c r="S3" s="90"/>
+      <c r="T3" s="90"/>
+      <c r="U3" s="90"/>
+      <c r="V3" s="90"/>
+      <c r="W3" s="90"/>
+      <c r="X3" s="90"/>
+      <c r="Y3" s="90"/>
+      <c r="Z3" s="90"/>
+      <c r="AA3" s="90"/>
+      <c r="AB3" s="90"/>
+      <c r="AC3" s="90"/>
+      <c r="AD3" s="90"/>
+      <c r="AE3" s="90"/>
+      <c r="AF3" s="90"/>
+      <c r="AG3" s="90"/>
+      <c r="AH3" s="90"/>
+      <c r="AI3" s="90"/>
+      <c r="AJ3" s="90"/>
+      <c r="AK3" s="90"/>
+      <c r="AL3" s="90"/>
+      <c r="AM3" s="90"/>
+      <c r="AN3" s="90"/>
+      <c r="AO3" s="90"/>
+      <c r="AP3" s="90"/>
+      <c r="AQ3" s="90"/>
+      <c r="AR3" s="90"/>
+      <c r="AS3" s="90"/>
+      <c r="AT3" s="90"/>
+      <c r="AU3" s="91"/>
     </row>
     <row r="4" spans="1:47" x14ac:dyDescent="0.2">
-      <c r="A4" s="81" t="s">
+      <c r="A4" s="82" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="82"/>
-      <c r="C4" s="83" t="s">
+      <c r="B4" s="83"/>
+      <c r="C4" s="84" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="84"/>
-      <c r="E4" s="84"/>
-      <c r="F4" s="84"/>
-      <c r="G4" s="84"/>
-      <c r="H4" s="84"/>
-      <c r="I4" s="84"/>
-      <c r="J4" s="84"/>
-      <c r="K4" s="84"/>
-      <c r="L4" s="84"/>
-      <c r="M4" s="84"/>
-      <c r="N4" s="84"/>
-      <c r="O4" s="84"/>
-      <c r="P4" s="84"/>
-      <c r="Q4" s="84"/>
-      <c r="R4" s="84"/>
-      <c r="S4" s="84"/>
-      <c r="T4" s="84"/>
-      <c r="U4" s="84"/>
-      <c r="V4" s="84"/>
-      <c r="W4" s="84"/>
-      <c r="X4" s="84"/>
-      <c r="Y4" s="84"/>
-      <c r="Z4" s="84"/>
-      <c r="AA4" s="84"/>
-      <c r="AB4" s="84"/>
-      <c r="AC4" s="84"/>
-      <c r="AD4" s="84"/>
-      <c r="AE4" s="84"/>
-      <c r="AF4" s="84"/>
-      <c r="AG4" s="84"/>
-      <c r="AH4" s="84"/>
-      <c r="AI4" s="84"/>
-      <c r="AJ4" s="84"/>
-      <c r="AK4" s="84"/>
-      <c r="AL4" s="84"/>
-      <c r="AM4" s="84"/>
-      <c r="AN4" s="84"/>
-      <c r="AO4" s="84"/>
-      <c r="AP4" s="84"/>
-      <c r="AQ4" s="84"/>
-      <c r="AR4" s="84"/>
-      <c r="AS4" s="84"/>
-      <c r="AT4" s="84"/>
-      <c r="AU4" s="85"/>
+      <c r="D4" s="85"/>
+      <c r="E4" s="85"/>
+      <c r="F4" s="85"/>
+      <c r="G4" s="85"/>
+      <c r="H4" s="85"/>
+      <c r="I4" s="85"/>
+      <c r="J4" s="85"/>
+      <c r="K4" s="85"/>
+      <c r="L4" s="85"/>
+      <c r="M4" s="85"/>
+      <c r="N4" s="85"/>
+      <c r="O4" s="85"/>
+      <c r="P4" s="85"/>
+      <c r="Q4" s="85"/>
+      <c r="R4" s="85"/>
+      <c r="S4" s="85"/>
+      <c r="T4" s="85"/>
+      <c r="U4" s="85"/>
+      <c r="V4" s="85"/>
+      <c r="W4" s="85"/>
+      <c r="X4" s="85"/>
+      <c r="Y4" s="85"/>
+      <c r="Z4" s="85"/>
+      <c r="AA4" s="85"/>
+      <c r="AB4" s="85"/>
+      <c r="AC4" s="85"/>
+      <c r="AD4" s="85"/>
+      <c r="AE4" s="85"/>
+      <c r="AF4" s="85"/>
+      <c r="AG4" s="85"/>
+      <c r="AH4" s="85"/>
+      <c r="AI4" s="85"/>
+      <c r="AJ4" s="85"/>
+      <c r="AK4" s="85"/>
+      <c r="AL4" s="85"/>
+      <c r="AM4" s="85"/>
+      <c r="AN4" s="85"/>
+      <c r="AO4" s="85"/>
+      <c r="AP4" s="85"/>
+      <c r="AQ4" s="85"/>
+      <c r="AR4" s="85"/>
+      <c r="AS4" s="85"/>
+      <c r="AT4" s="85"/>
+      <c r="AU4" s="86"/>
     </row>
     <row r="5" spans="1:47" x14ac:dyDescent="0.2">
-      <c r="A5" s="81" t="s">
+      <c r="A5" s="82" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="82"/>
-      <c r="C5" s="83" t="s">
+      <c r="B5" s="83"/>
+      <c r="C5" s="84" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="84"/>
-      <c r="E5" s="84"/>
-      <c r="F5" s="84"/>
-      <c r="G5" s="84"/>
-      <c r="H5" s="84"/>
-      <c r="I5" s="84"/>
-      <c r="J5" s="84"/>
-      <c r="K5" s="84"/>
-      <c r="L5" s="84"/>
-      <c r="M5" s="84"/>
-      <c r="N5" s="84"/>
-      <c r="O5" s="84"/>
-      <c r="P5" s="84"/>
-      <c r="Q5" s="84"/>
-      <c r="R5" s="84"/>
-      <c r="S5" s="84"/>
-      <c r="T5" s="84"/>
-      <c r="U5" s="84"/>
-      <c r="V5" s="84"/>
-      <c r="W5" s="84"/>
-      <c r="X5" s="84"/>
-      <c r="Y5" s="84"/>
-      <c r="Z5" s="84"/>
-      <c r="AA5" s="84"/>
-      <c r="AB5" s="84"/>
-      <c r="AC5" s="84"/>
-      <c r="AD5" s="84"/>
-      <c r="AE5" s="84"/>
-      <c r="AF5" s="84"/>
-      <c r="AG5" s="84"/>
-      <c r="AH5" s="84"/>
-      <c r="AI5" s="84"/>
-      <c r="AJ5" s="84"/>
-      <c r="AK5" s="84"/>
-      <c r="AL5" s="84"/>
-      <c r="AM5" s="84"/>
-      <c r="AN5" s="84"/>
-      <c r="AO5" s="84"/>
-      <c r="AP5" s="84"/>
-      <c r="AQ5" s="84"/>
-      <c r="AR5" s="84"/>
-      <c r="AS5" s="84"/>
-      <c r="AT5" s="84"/>
-      <c r="AU5" s="85"/>
+      <c r="D5" s="85"/>
+      <c r="E5" s="85"/>
+      <c r="F5" s="85"/>
+      <c r="G5" s="85"/>
+      <c r="H5" s="85"/>
+      <c r="I5" s="85"/>
+      <c r="J5" s="85"/>
+      <c r="K5" s="85"/>
+      <c r="L5" s="85"/>
+      <c r="M5" s="85"/>
+      <c r="N5" s="85"/>
+      <c r="O5" s="85"/>
+      <c r="P5" s="85"/>
+      <c r="Q5" s="85"/>
+      <c r="R5" s="85"/>
+      <c r="S5" s="85"/>
+      <c r="T5" s="85"/>
+      <c r="U5" s="85"/>
+      <c r="V5" s="85"/>
+      <c r="W5" s="85"/>
+      <c r="X5" s="85"/>
+      <c r="Y5" s="85"/>
+      <c r="Z5" s="85"/>
+      <c r="AA5" s="85"/>
+      <c r="AB5" s="85"/>
+      <c r="AC5" s="85"/>
+      <c r="AD5" s="85"/>
+      <c r="AE5" s="85"/>
+      <c r="AF5" s="85"/>
+      <c r="AG5" s="85"/>
+      <c r="AH5" s="85"/>
+      <c r="AI5" s="85"/>
+      <c r="AJ5" s="85"/>
+      <c r="AK5" s="85"/>
+      <c r="AL5" s="85"/>
+      <c r="AM5" s="85"/>
+      <c r="AN5" s="85"/>
+      <c r="AO5" s="85"/>
+      <c r="AP5" s="85"/>
+      <c r="AQ5" s="85"/>
+      <c r="AR5" s="85"/>
+      <c r="AS5" s="85"/>
+      <c r="AT5" s="85"/>
+      <c r="AU5" s="86"/>
     </row>
     <row r="6" spans="1:47" x14ac:dyDescent="0.2">
-      <c r="A6" s="81" t="s">
+      <c r="A6" s="82" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="82"/>
-      <c r="C6" s="83" t="s">
+      <c r="B6" s="83"/>
+      <c r="C6" s="84" t="s">
         <v>44</v>
       </c>
-      <c r="D6" s="84"/>
-      <c r="E6" s="84"/>
-      <c r="F6" s="84"/>
-      <c r="G6" s="84"/>
-      <c r="H6" s="84"/>
-      <c r="I6" s="84"/>
-      <c r="J6" s="84"/>
-      <c r="K6" s="84"/>
-      <c r="L6" s="84"/>
-      <c r="M6" s="84"/>
-      <c r="N6" s="84"/>
-      <c r="O6" s="84"/>
-      <c r="P6" s="84"/>
-      <c r="Q6" s="84"/>
-      <c r="R6" s="84"/>
-      <c r="S6" s="84"/>
-      <c r="T6" s="84"/>
-      <c r="U6" s="84"/>
-      <c r="V6" s="84"/>
-      <c r="W6" s="84"/>
-      <c r="X6" s="84"/>
-      <c r="Y6" s="84"/>
-      <c r="Z6" s="84"/>
-      <c r="AA6" s="84"/>
-      <c r="AB6" s="84"/>
-      <c r="AC6" s="84"/>
-      <c r="AD6" s="84"/>
-      <c r="AE6" s="84"/>
-      <c r="AF6" s="84"/>
-      <c r="AG6" s="84"/>
-      <c r="AH6" s="84"/>
-      <c r="AI6" s="84"/>
-      <c r="AJ6" s="84"/>
-      <c r="AK6" s="84"/>
-      <c r="AL6" s="84"/>
-      <c r="AM6" s="84"/>
-      <c r="AN6" s="84"/>
-      <c r="AO6" s="84"/>
-      <c r="AP6" s="84"/>
-      <c r="AQ6" s="84"/>
-      <c r="AR6" s="84"/>
-      <c r="AS6" s="84"/>
-      <c r="AT6" s="84"/>
-      <c r="AU6" s="85"/>
+      <c r="D6" s="85"/>
+      <c r="E6" s="85"/>
+      <c r="F6" s="85"/>
+      <c r="G6" s="85"/>
+      <c r="H6" s="85"/>
+      <c r="I6" s="85"/>
+      <c r="J6" s="85"/>
+      <c r="K6" s="85"/>
+      <c r="L6" s="85"/>
+      <c r="M6" s="85"/>
+      <c r="N6" s="85"/>
+      <c r="O6" s="85"/>
+      <c r="P6" s="85"/>
+      <c r="Q6" s="85"/>
+      <c r="R6" s="85"/>
+      <c r="S6" s="85"/>
+      <c r="T6" s="85"/>
+      <c r="U6" s="85"/>
+      <c r="V6" s="85"/>
+      <c r="W6" s="85"/>
+      <c r="X6" s="85"/>
+      <c r="Y6" s="85"/>
+      <c r="Z6" s="85"/>
+      <c r="AA6" s="85"/>
+      <c r="AB6" s="85"/>
+      <c r="AC6" s="85"/>
+      <c r="AD6" s="85"/>
+      <c r="AE6" s="85"/>
+      <c r="AF6" s="85"/>
+      <c r="AG6" s="85"/>
+      <c r="AH6" s="85"/>
+      <c r="AI6" s="85"/>
+      <c r="AJ6" s="85"/>
+      <c r="AK6" s="85"/>
+      <c r="AL6" s="85"/>
+      <c r="AM6" s="85"/>
+      <c r="AN6" s="85"/>
+      <c r="AO6" s="85"/>
+      <c r="AP6" s="85"/>
+      <c r="AQ6" s="85"/>
+      <c r="AR6" s="85"/>
+      <c r="AS6" s="85"/>
+      <c r="AT6" s="85"/>
+      <c r="AU6" s="86"/>
     </row>
     <row r="7" spans="1:47" ht="126" x14ac:dyDescent="0.2">
-      <c r="A7" s="86" t="s">
+      <c r="A7" s="87" t="s">
         <v>45</v>
       </c>
-      <c r="B7" s="87"/>
+      <c r="B7" s="88"/>
       <c r="C7" s="8" t="s">
         <v>46</v>
       </c>
@@ -8764,7 +8764,7 @@
       <c r="D22" s="76">
         <v>175287.99999999997</v>
       </c>
-      <c r="E22" s="91" t="s">
+      <c r="E22" s="92" t="s">
         <v>215</v>
       </c>
       <c r="F22" s="46" t="s">
@@ -8784,7 +8784,7 @@
       <c r="D23" s="61">
         <v>25127</v>
       </c>
-      <c r="E23" s="91"/>
+      <c r="E23" s="92"/>
       <c r="F23" s="46" t="s">
         <v>176</v>
       </c>
@@ -9058,7 +9058,7 @@
         <f>'OECD TTL'!W49*10^6*About!$A$30*('BR Data for ISIC Splits'!R6/SUM('BR Data for ISIC Splits'!P6:R6))</f>
         <v>57763254487.389854</v>
       </c>
-      <c r="AC2" s="92">
+      <c r="AC2" s="81">
         <f>'OECD TTL'!X30*10^6*About!A30</f>
         <v>132321902.64833325</v>
       </c>

</xml_diff>